<commit_message>
Add confirmation modals for debt actions in DebtPage
Replaced window.confirm with custom modals for deleting, closing, and saving debts. Introduced new state variables to manage modal visibility and context. Updated action handlers to use these modals, enhancing user experience and consistency. Also adjusted interest calculation to use end-of-day for current date.
</commit_message>
<xml_diff>
--- a/Check list.xlsx
+++ b/Check list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\ManagementFincance\FinanceManagementApplication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C98C008D-87D6-435F-89F5-AC7FA61311F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A7922F-CB94-4668-A270-1DF539F3EA18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7003FEB6-D9D2-4C85-95CB-1CF7FE35B8F1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="84">
   <si>
     <t>Account already exists</t>
   </si>
@@ -57,12 +57,6 @@
 2. Enter email already exists
 3. Warning email is registered
 4. Keep in register page</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>It didn't keep in register page</t>
   </si>
   <si>
     <t>Login</t>
@@ -73,6 +67,300 @@
 Password: 123456
 2. Choose Login
 3. Show Dashboard page</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Tổng giá trị tài sản gốc hiển thị đúng giá trị</t>
+  </si>
+  <si>
+    <t>Net worth hiển thị dúng giá trị</t>
+  </si>
+  <si>
+    <t>Original Value</t>
+  </si>
+  <si>
+    <t>Net worth</t>
+  </si>
+  <si>
+    <t>Tỉ lệ % của net worth hiển thị đúng giá trị</t>
+  </si>
+  <si>
+    <t>Tiến độ mục tiêu</t>
+  </si>
+  <si>
+    <t>Tiến độ mục tiêu phải hiển thị bao gồm những yếu tố sau:
+Thông tin mục tiêu gần nhất
+Tên
+Thanh tiến độ hoàn thành
+Số ngày còn lại
+Tỉ lệ hoàn thành</t>
+  </si>
+  <si>
+    <t>Cash Flow Growth</t>
+  </si>
+  <si>
+    <t>Theo năm:
+Hiện thị toàn bộ giá trị của các năm</t>
+  </si>
+  <si>
+    <t>Theo tháng:
+Hiển thị toàn bộ giá trị của toàn bộ tháng trong năm đó.
+Nếu thời điểm xem là năm hiện tại thì lấy các tháng cho tới thời điệm hiện tại</t>
+  </si>
+  <si>
+    <t>Theo 12 tháng:
+Hiển thị toàn bộ giá trị tàn sản tính từ thời điểm hiện tại cho tới 12 tháng về trước.
+Nếu từ thời điểm hiện tại tới 12 tháng về trước không có đủ toàn bộ data của 12 tháng thì lấy data tháng có data xa nhất không qua 12 tháng</t>
+  </si>
+  <si>
+    <t>Phân bổ tài sản</t>
+  </si>
+  <si>
+    <t>Với tổng quan:
+Chỉ hiển thị tài sản tiết kiệm và đầu tư
+Đảm bảo tổng số tài sản hiện thị đúng đơn vị viết tắt
+Đẳm bảo bar chart hiển thị đúng</t>
+  </si>
+  <si>
+    <t>Với chi tiết:
+Hiển thị toàn bộ tại sảng đang có
+Đảm bảo tổng số tài sản hiện thị đúng đơn vị viết tắt
+Đẳm bảo bar chart hiển thị đúng</t>
+  </si>
+  <si>
+    <t>Quản lý tài sản</t>
+  </si>
+  <si>
+    <t>bảng quản lý tài sản chi tiết</t>
+  </si>
+  <si>
+    <t>Hiển thị toàn bộ tài sản hiện có của user. Phân chia đúng tài sản tiết kiệm và tài sản đầu tư
+STT
+Tên tài sản
+Vốn ban đầu
+Giá trị hiện tại
+Lợi nhuận
+Tỷ suất
+Ngày cập nhật
+Hành động</t>
+  </si>
+  <si>
+    <t>Thêm tài sản</t>
+  </si>
+  <si>
+    <t>Hiển thị pop-up khi nhấn thêm tài sản, bao gồm các thông tin
+- Tên tài sản
+- Vốn ban đầu
+- Giá trị hiện tại
+Phân loại (tiết kiệm, đầu tư)</t>
+  </si>
+  <si>
+    <t>Bắt buộc điền tên tài sản</t>
+  </si>
+  <si>
+    <t>Điền toàn bộ thông tin và lưu thành công</t>
+  </si>
+  <si>
+    <t>Lưu thông tin</t>
+  </si>
+  <si>
+    <t>Nhấn lưu thông tin
+Thông tin mới được lưu sẽ được cập nhật vào lịch sử lưu thông tin</t>
+  </si>
+  <si>
+    <t>Cập nhật tài sản</t>
+  </si>
+  <si>
+    <t>Chọn 1 tài sản bất kỳ và thay đổi thông tin
+Lưu thành công</t>
+  </si>
+  <si>
+    <t>Chọn 1 tài sản bất kỳ và xóa toàn bộ tên tài sản
+Sau khi nhấn lưu thông tin thì hiện bắt buộc phải nhập</t>
+  </si>
+  <si>
+    <t>Chọn 1 tài sản bất kỳ và chọn sửa tài sản
+Nhấn button Hủy
+Thoát ra mà không làm thay đổi bất kỳ thông tin gì</t>
+  </si>
+  <si>
+    <t>Xóa tài sản</t>
+  </si>
+  <si>
+    <t>Nhấn xóa tài sản
+Hiện pop-up thông báo và cho phép xóa hay không
+Chọn Xóa, tài sản bị xóa</t>
+  </si>
+  <si>
+    <t>Nhấn xóa tài sản
+Hiện pop-up thông báo và cho phép xóa hay không
+Chọn Hủy, Tài sản không bị xóa, đảm bảo toàn bộ thông tin không đổi</t>
+  </si>
+  <si>
+    <t>Nếu tài sản lợi giá trị hiện tại là 0 thì đảm bảo tỷ suất là 0 (không hiển thị lỗi chia 0)</t>
+  </si>
+  <si>
+    <t>Lịch sử lưu thông tin</t>
+  </si>
+  <si>
+    <t>Lịch sử lưu thông tin phải hiển thị toàn bộ lịch sửa mà người dùng đã lưu theo thứ tự ngày lưu</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ record nào trong lịch sử lưu thông tin và nhấn Khôi phục
+Hiển thị đúng các thông tin của record đó lên bảng quản lý tài sản chi tiết</t>
+  </si>
+  <si>
+    <t>Phân bổ danh mục</t>
+  </si>
+  <si>
+    <t>Bảng phân bổ danh mục</t>
+  </si>
+  <si>
+    <t>Nhấn tab phân bổ danh mục
+Hiển thị toàn bộ phân bổ đã lưu trước đó</t>
+  </si>
+  <si>
+    <t>Nhập thu nhập</t>
+  </si>
+  <si>
+    <t>Nhập thu nhập, tự động phân bổ số tiền vào các danh mục đưa vào thiết lập đã được thiết lập trước đó</t>
+  </si>
+  <si>
+    <t>Nhập số tiền cần giảm</t>
+  </si>
+  <si>
+    <t>Số tiền giảm sẽ được phân bổ dựa vào tỉ lệ phân trăm danh mục đã được lưu trước đó</t>
+  </si>
+  <si>
+    <t>Loại trừ</t>
+  </si>
+  <si>
+    <t>Khi nhấn loại trừ, danh mục đó sẽ không bị giảm tiền. Số tiền đó sẽ được phân bổ vào các danh mục  còn lại</t>
+  </si>
+  <si>
+    <t>Áp dụng</t>
+  </si>
+  <si>
+    <t>Nếu danh mục được kết nối với tài sản thì phần áp dụng sẽ sáng lên
+Khi nhấn áp dụng, tiền sẽ được cộng thẳng vào tài sản (vốn ban đầu và giá trị hiện tại) đã được liên kết sẵn</t>
+  </si>
+  <si>
+    <t>Nếu thu nhập là 0 thì phải đẳm bảo giá trị trong bảng phân bổ đều là 0</t>
+  </si>
+  <si>
+    <t>Thiết lập mới</t>
+  </si>
+  <si>
+    <t>Lưu tiết lập</t>
+  </si>
+  <si>
+    <t>Vào thiết lập mới
+Khi nhấn Hủy thì quay trở lại Phân bổ Danh mục</t>
+  </si>
+  <si>
+    <t>Vào thiết lập mới
+Nhấn lưu thiết lập sẽ lưu toàn bộ tiết lập trong bảng thiết lập vào lịch sử (thiết lập sẽ không lưu tài sản đã liên kết)
+- Thông tin được lưu bao gồm phaan6 bổ gốc, các danh mục trong bảng phân bổ</t>
+  </si>
+  <si>
+    <t>Vào thiết lập mới
+Hiển thị toàn bộ thông tin của bảng thiết lập đã được user lưu
+- Phân loại: Bao gồm sinh hoạt, tiết kiệm và đầu tư
+- Tên danh mục sẽ hiển thị tên và tài sản liên kết
+- Số tiền phân bổ
+- Tỉ trọng</t>
+  </si>
+  <si>
+    <t>Vào thiết lập mới
+Hiển thị toàn bộ thông tin của bảng thiết lập đã được user lưu
+Chỉnh sửa số tiền phân bổ (đảm bảo số tiền hợp lệ và không được quá số tiền phân bổ gốc)</t>
+  </si>
+  <si>
+    <t>Vào thiết lập mới
+Chọn một danh mục bất kỳ và chọn liên kết tài sản bất kỳ
+Nhấn lưu thiết lập
+Refresh lại để kiểm tra danh mục đó liên kết tài sản đúng hay không
+Quay lại tab phân bổ danh mục xem tài sản đó đã được ký hiệu là liên kết hay chưa</t>
+  </si>
+  <si>
+    <t>Xóa danh mục trong phân bổ danh mục</t>
+  </si>
+  <si>
+    <t>Vào thiết lập mới
+Xóa danh mục bất kỳ 
+Hiện popup hỏi xóa hay không
+Khi nhấn xóa và chọn lưu thiết lập, kiểm tra xem danh mục đó đã được xóa trong phân bổ danh mục và thiết lập mới hay chưa</t>
+  </si>
+  <si>
+    <t>Lịch sử phân bổ</t>
+  </si>
+  <si>
+    <t>Hiển thị toàn bộ lịch sử đã được lưu và xếp theo thời gian</t>
+  </si>
+  <si>
+    <t>Khôi phục danh mục</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ record nào trong lịch sử phân bổ sau đó nhấn khôi phục
+Đảm bảo các giá trị như phân bổ gốc và các danh mục được khôi phục đúng</t>
+  </si>
+  <si>
+    <t>Mục tiêu</t>
+  </si>
+  <si>
+    <t>Dashboard thiết lập thông tin</t>
+  </si>
+  <si>
+    <t>Hiển thị đúng tổng số mục tiêu
+Hiện thị đúng tài sản hiện có
+Hiển thị đúng mục tiêu gần nhất</t>
+  </si>
+  <si>
+    <t>Thêm mục tiêu</t>
+  </si>
+  <si>
+    <t>Để rỗng tên mục tiêu -&gt; không cho tạo</t>
+  </si>
+  <si>
+    <t>Điền input, để trống ngày đến hạn -&gt; không cho tạo</t>
+  </si>
+  <si>
+    <t>Điền input, điền giá trị tiền âm -&gt; không cho tạo</t>
+  </si>
+  <si>
+    <t>Bảng mục tiêu</t>
+  </si>
+  <si>
+    <t>Nếu tài sản hiện có &lt; số tiền mục tiêu và vẫn trong hạn -&gt; báo đang thực hiện</t>
+  </si>
+  <si>
+    <t>Nếu tài sản hiện có &gt; số tiền mục tiêu (trong hạn thực hiện) -&gt; Báo thành công</t>
+  </si>
+  <si>
+    <t>Điền toàn bộ input hợp lệ -&gt; cho phép tạo</t>
+  </si>
+  <si>
+    <t>Điền toàn bộ input, ngày bắt đầu lớn hơn ngày bắt đầu -&gt; không cho phép tạo</t>
+  </si>
+  <si>
+    <t>Nếu tài sản hiện có &lt; số tiền mục tiêu và không trong hạn -&gt; báo thật bại</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ mục tiêu nào đang trong trạng thái đang thực hiện -&gt; chọn hủy -&gt; chuyển sang trạng thái đã hủy</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ mục tiêu nào đang trong trạng thái chưa bắt đầu -&gt; nhấn bắt đầu -&gt; chuyển sang trạng thái đang thực hiện</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ mục tiêu nào -&gt; chọn hành động xóa -&gt; refresh lại page để kiểm tra đảm bảo mục tiêu đó đã bị xóa</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ mục tiêu nào -&gt; chọn hành động chỉnh sửa -&gt; sau khi chỉnh sửa thì cập nhật toàn bộ trạng thái phù hợp với điều kiện chỉnh sửa
+Nếu ngày kết thúc &lt; ngày hiện tại và số tiền mục tiêu &lt; số tiền hiện tại -&gt; Thất bại
+Nếu ngày bắt đầu &gt; ngày hiện tại -&gt; trạng thái chưa bắt đầu
+Nếu ngày bắt đầu &lt; ngày hiện tại: Kiểm tra điều kiện giá nếu tiền mục tiêu &lt; tiền hiện tại -&gt; trạng thái đang thực hiện, ngược lại là thành công</t>
   </si>
 </sst>
 </file>
@@ -96,7 +384,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -119,11 +407,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -131,6 +456,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -466,53 +803,837 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8EE68B3-A339-4AF8-A1DF-6D8E15A895EC}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="55.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="26.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="98.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:5" ht="98.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="4"/>
+      <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="4"/>
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="D4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>3</v>
-      </c>
+      <c r="D5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="6"/>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="6"/>
+      <c r="B10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A11" s="6"/>
+      <c r="B11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="6"/>
+      <c r="B12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="7"/>
+      <c r="B13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" ht="150" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+      <c r="B15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="6"/>
+      <c r="B16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="6"/>
+      <c r="B17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="6"/>
+      <c r="B18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="6"/>
+      <c r="B19" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="6"/>
+      <c r="B20" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="6"/>
+      <c r="B21" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="6"/>
+      <c r="B23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="6"/>
+      <c r="B25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26" s="7"/>
+      <c r="B26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="6"/>
+      <c r="B28" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="6"/>
+      <c r="B29" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="6"/>
+      <c r="B30" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="6"/>
+      <c r="B31" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A32" s="6"/>
+      <c r="B32" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="6"/>
+      <c r="B33" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A34" s="6"/>
+      <c r="B34" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A35" s="6"/>
+      <c r="B35" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A36" s="6"/>
+      <c r="B36" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A37" s="6"/>
+      <c r="B37" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A38" s="6"/>
+      <c r="B38" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="6"/>
+      <c r="B39" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A40" s="7"/>
+      <c r="B40" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="6"/>
+      <c r="B42" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="6"/>
+      <c r="B43" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="6"/>
+      <c r="B44" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E44" s="2"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="6"/>
+      <c r="B45" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A46" s="6"/>
+      <c r="B46" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" s="6"/>
+      <c r="B47" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="6"/>
+      <c r="B48" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A49" s="6"/>
+      <c r="B49" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="6"/>
+      <c r="B50" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="6"/>
+      <c r="B51" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E51" s="2"/>
+    </row>
+    <row r="52" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="6"/>
+      <c r="B52" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E52" s="2"/>
+    </row>
+    <row r="53" spans="1:5" ht="135" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="2"/>
+      <c r="B65" s="2"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="2"/>
+      <c r="B66" s="2"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="2"/>
+      <c r="B68" s="2"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="2"/>
+      <c r="E70" s="2"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A13"/>
+    <mergeCell ref="A14:A26"/>
+    <mergeCell ref="A27:A40"/>
+    <mergeCell ref="A41:A53"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add delete support for asset/allocation history records
Implemented backend and frontend logic to delete asset and allocation history records. Added new API endpoints and repository methods for deletion. Updated React components and services to support deleting history entries and refreshing UI state. Improved allocation sorting in demo mode.
</commit_message>
<xml_diff>
--- a/Check list.xlsx
+++ b/Check list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\ManagementFincance\FinanceManagementApplication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A7922F-CB94-4668-A270-1DF539F3EA18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB5F4E5-723C-47A7-9BE2-3B1DA69161CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7003FEB6-D9D2-4C85-95CB-1CF7FE35B8F1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="104">
   <si>
     <t>Account already exists</t>
   </si>
@@ -361,6 +361,66 @@
 Nếu ngày kết thúc &lt; ngày hiện tại và số tiền mục tiêu &lt; số tiền hiện tại -&gt; Thất bại
 Nếu ngày bắt đầu &gt; ngày hiện tại -&gt; trạng thái chưa bắt đầu
 Nếu ngày bắt đầu &lt; ngày hiện tại: Kiểm tra điều kiện giá nếu tiền mục tiêu &lt; tiền hiện tại -&gt; trạng thái đang thực hiện, ngược lại là thành công</t>
+  </si>
+  <si>
+    <t>Quản lý nợ</t>
+  </si>
+  <si>
+    <t>Thông tin</t>
+  </si>
+  <si>
+    <t>Hiển thị đúng tổng số nợ</t>
+  </si>
+  <si>
+    <t>Hiển thị đúng giá trị nợ còn lại</t>
+  </si>
+  <si>
+    <t>Hiển thị đúng giá trị nợ đã trả</t>
+  </si>
+  <si>
+    <t>Hiển thị đúng khoản nợ sắp hết hạn</t>
+  </si>
+  <si>
+    <t>Lịch sử thanh toán</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ khoản nợ nào -&gt; nhấn vào để hiển thị toàn bộ lịch sử thanh toán</t>
+  </si>
+  <si>
+    <t>Thêm sổ nợ</t>
+  </si>
+  <si>
+    <t>Nhập thông tin hợp lệ -&gt; thêm -&gt; tạo thành công</t>
+  </si>
+  <si>
+    <t>Thanh toán</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ khoản nợ đang trong trạng thái đang vay -&gt; Chọn thanh toán -&gt; Nhập giá trị -&gt; Xác nhận -&gt; Kiểm tra lịch sử, số tiền đã trả đúng, số tiền còn lại đúng</t>
+  </si>
+  <si>
+    <t>Sửa</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ khoản nợ đang trong trạng thái đang vay -&gt; Chọn sửa -&gt; sửa thành giá trị hợp lý -&gt; Lưu -&gt; các giá trị cập nhật hợp lệ</t>
+  </si>
+  <si>
+    <t>Đóng sổ</t>
+  </si>
+  <si>
+    <t>Xóa</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ khoản nợ đang trong trạng thái đang vay -&gt; Đóng sổ -&gt; Popup thông báo hiện lên -&gt; Khoản nợ được chuyển thành trạng thái đóng</t>
+  </si>
+  <si>
+    <t>Chọn bất kỳ khoản nợ-&gt; Xóa -&gt; Popup thông báo hiện lên -&gt; Khoản nợ được xóa thành công</t>
+  </si>
+  <si>
+    <t>Tiền lãi</t>
+  </si>
+  <si>
+    <t>Kiểm tra xem tiền lãi được tính toán đúng hay không</t>
   </si>
 </sst>
 </file>
@@ -448,7 +508,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -468,6 +528,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1500,133 +1564,202 @@
       <c r="E53" s="2"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="2"/>
+      <c r="A54" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E54" s="2"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="2"/>
+      <c r="A55" s="6"/>
+      <c r="B55" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E55" s="2"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="2"/>
+      <c r="A56" s="6"/>
+      <c r="B56" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E56" s="2"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="2"/>
+      <c r="A57" s="6"/>
+      <c r="B57" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="2"/>
+    <row r="58" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="6"/>
+      <c r="B58" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E58" s="2"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="2"/>
+      <c r="A59" s="6"/>
+      <c r="B59" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E59" s="2"/>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="3"/>
-      <c r="D60" s="2"/>
+    <row r="60" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A60" s="6"/>
+      <c r="B60" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E60" s="2"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="3"/>
-      <c r="D61" s="2"/>
+    <row r="61" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A61" s="6"/>
+      <c r="B61" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E61" s="2"/>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="2"/>
+    <row r="62" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A62" s="6"/>
+      <c r="B62" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E62" s="2"/>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="2"/>
+    <row r="63" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="6"/>
+      <c r="B63" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E63" s="2"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="2"/>
+      <c r="A64" s="7"/>
+      <c r="B64" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="E64" s="2"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="3"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
+      <c r="A65" s="8"/>
+      <c r="B65" s="8"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="8"/>
+      <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="3"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
+      <c r="A66" s="8"/>
+      <c r="B66" s="8"/>
+      <c r="C66" s="9"/>
+      <c r="D66" s="8"/>
+      <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
+      <c r="A67" s="8"/>
+      <c r="B67" s="8"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="8"/>
+      <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
+      <c r="A68" s="8"/>
+      <c r="B68" s="8"/>
+      <c r="C68" s="9"/>
+      <c r="D68" s="8"/>
+      <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
+      <c r="A69" s="8"/>
+      <c r="B69" s="8"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="8"/>
+      <c r="E69" s="8"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
+      <c r="A70" s="8"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
+      <c r="A71" s="8"/>
+      <c r="B71" s="8"/>
+      <c r="C71" s="9"/>
+      <c r="D71" s="8"/>
+      <c r="E71" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A54:A64"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A5:A13"/>
     <mergeCell ref="A14:A26"/>

</xml_diff>